<commit_message>
RCA flow change of tbab names
</commit_message>
<xml_diff>
--- a/streamlit_rca_code/data/Network_Link_CRC.xlsx
+++ b/streamlit_rca_code/data/Network_Link_CRC.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="8000" firstSheet="2" activeTab="1"/>
+    <workbookView windowWidth="20490" windowHeight="7500" firstSheet="2" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -202,13 +202,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
       <t>[</t>
     </r>
     <r>
@@ -218,7 +211,7 @@
         <rFont val="Consolas"/>
         <charset val="134"/>
       </rPr>
-      <t>"High crc arror detected on Gi0/1"]</t>
+      <t>"High crc error detected on Gi0/1"]</t>
     </r>
   </si>
   <si>
@@ -239,10 +232,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -739,16 +732,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -918,7 +911,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1252,21 +1245,21 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="21.0909090909091" customWidth="1"/>
-    <col min="3" max="3" width="8.90909090909091" customWidth="1"/>
-    <col min="4" max="4" width="9.81818181818182" customWidth="1"/>
-    <col min="5" max="5" width="12.2727272727273" customWidth="1"/>
-    <col min="6" max="6" width="13.7272727272727" customWidth="1"/>
-    <col min="7" max="7" width="7.81818181818182" customWidth="1"/>
-    <col min="8" max="8" width="13.1818181818182" customWidth="1"/>
-    <col min="9" max="9" width="18.3636363636364" customWidth="1"/>
-    <col min="10" max="10" width="9.18181818181818" customWidth="1"/>
-    <col min="11" max="11" width="12.6363636363636" customWidth="1"/>
-    <col min="12" max="12" width="11.1818181818182" customWidth="1"/>
+    <col min="1" max="2" width="21.0952380952381" customWidth="1"/>
+    <col min="3" max="3" width="8.90476190476191" customWidth="1"/>
+    <col min="4" max="4" width="9.81904761904762" customWidth="1"/>
+    <col min="5" max="5" width="12.2761904761905" customWidth="1"/>
+    <col min="6" max="6" width="13.7238095238095" customWidth="1"/>
+    <col min="7" max="7" width="7.81904761904762" customWidth="1"/>
+    <col min="8" max="8" width="13.1809523809524" customWidth="1"/>
+    <col min="9" max="9" width="18.3619047619048" customWidth="1"/>
+    <col min="10" max="10" width="9.18095238095238" customWidth="1"/>
+    <col min="11" max="11" width="12.6380952380952" customWidth="1"/>
+    <col min="12" max="12" width="11.1809523809524" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="21.0909090909091" customWidth="1"/>
+    <col min="14" max="14" width="21.0952380952381" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="1" spans="1:16">
@@ -1319,7 +1312,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -1351,7 +1344,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1383,7 +1376,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1415,7 +1408,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>22</v>
       </c>
@@ -1447,7 +1440,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -1479,7 +1472,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1505,7 +1498,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1531,7 +1524,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:16">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1557,7 +1550,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1583,7 +1576,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1619,15 +1612,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:G6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="1" width="22.4545454545455" customWidth="1"/>
-    <col min="2" max="2" width="23.3636363636364" customWidth="1"/>
-    <col min="5" max="5" width="20.0909090909091" customWidth="1"/>
-    <col min="7" max="7" width="20.6363636363636" customWidth="1"/>
+    <col min="1" max="1" width="22.4571428571429" customWidth="1"/>
+    <col min="2" max="2" width="23.3619047619048" customWidth="1"/>
+    <col min="5" max="5" width="20.0952380952381" customWidth="1"/>
+    <col min="7" max="7" width="20.6380952380952" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" spans="1:7">
+    <row r="1" ht="30" spans="1:7">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -1650,7 +1643,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="2" ht="29" spans="1:7">
+    <row r="2" ht="30" spans="1:7">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1696,7 +1689,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" ht="29" spans="1:7">
+    <row r="4" ht="30" spans="1:7">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -1719,7 +1712,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" ht="29" spans="1:7">
+    <row r="5" ht="30" spans="1:7">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -1775,12 +1768,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="2" width="19.4545454545455" customWidth="1"/>
-    <col min="3" max="3" width="19.6363636363636" customWidth="1"/>
-    <col min="4" max="4" width="65.4545454545455" customWidth="1"/>
-    <col min="5" max="5" width="41.1818181818182" customWidth="1"/>
+    <col min="1" max="2" width="19.4571428571429" customWidth="1"/>
+    <col min="3" max="3" width="19.6380952380952" customWidth="1"/>
+    <col min="4" max="4" width="65.4571428571429" customWidth="1"/>
+    <col min="5" max="5" width="41.1809523809524" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -1885,7 +1878,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="4:4">
+    <row r="7" spans="1:5">
       <c r="D7" s="3"/>
     </row>
   </sheetData>
@@ -1898,15 +1891,15 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:F2"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="5"/>
+  <sheetFormatPr defaultColWidth="8.72380952380952" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="1" width="24.1818181818182" customWidth="1"/>
-    <col min="2" max="2" width="21.8181818181818" customWidth="1"/>
-    <col min="3" max="3" width="23.9090909090909" customWidth="1"/>
-    <col min="6" max="6" width="72.3636363636364" customWidth="1"/>
+    <col min="1" max="1" width="24.1809523809524" customWidth="1"/>
+    <col min="2" max="2" width="21.8190476190476" customWidth="1"/>
+    <col min="3" max="3" width="23.9047619047619" customWidth="1"/>
+    <col min="6" max="6" width="72.3619047619048" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="29" spans="1:6">
+    <row r="1" ht="30" spans="1:6">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1956,7 +1949,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="8.72727272727273" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="2"/>
+  <sheetFormatPr defaultColWidth="8.72380952380952" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="2"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">

</xml_diff>